<commit_message>
Updating with local drive Created a cleaner version for running the model with different exposure scenarios Model parameters were not changed Model structure changed depending on the exposure scenario
</commit_message>
<xml_diff>
--- a/Input/Experimental.Plasma.PFOA.xlsx
+++ b/Input/Experimental.Plasma.PFOA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4.sharepoint.com/sites/PARCProjectChrysanthi-CChannel/Gedeelde documenten/C_Channel/CP_L_R/PARC_PFAS_PBPKmodel/Codes_PFAS_models/Chrysanthi_Pachoulide_2024_PFOA_oral_dermal_blood/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4.sharepoint.com/sites/PARCProjectChrysanthi-CChannel/Gedeelde documenten/C_Channel/CP_L_R/PARC_PFOA_mechanistic/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{158E748D-52F5-4ADD-A8A4-8337E2F609AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:40009_{158E748D-52F5-4ADD-A8A4-8337E2F609AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87DA9605-6E84-4AFA-8328-9DD6F70F672A}"/>
   <bookViews>
-    <workbookView xWindow="31635" yWindow="2775" windowWidth="21600" windowHeight="11295"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experimental.Plasma.PFOA" sheetId="1" r:id="rId1"/>
@@ -433,7 +433,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -913,7 +913,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -973,9 +973,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1013,7 +1013,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1119,7 +1119,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1261,742 +1261,745 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B91"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="8.7265625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
         <v>1</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>1125</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>1375</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="1">
         <v>2</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="1">
         <v>3</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" s="1">
         <v>4</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" s="1">
         <v>5</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="1">
         <v>6</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="1">
         <v>7</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="1">
         <v>8</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="1">
         <v>9</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="1">
         <v>10</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="1">
         <v>11</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="1">
         <v>12</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="1">
         <v>13</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="1">
         <v>14</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="1">
         <v>16</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="1">
         <v>18</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" s="1">
         <v>20</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="1">
         <v>22</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" s="1">
         <v>24</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
         <v>28</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" s="1">
         <v>32</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="1">
         <v>36</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" s="1">
         <v>40</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="1">
         <v>44</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" s="1">
         <v>51</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" s="1">
         <v>58</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" s="1">
         <v>65</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" s="1">
         <v>72</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" s="1">
         <v>86</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" s="1">
         <v>100</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" s="1">
         <v>114</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" s="1">
         <v>128</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" s="1">
         <v>142</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" s="1">
         <v>170</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" s="1">
         <v>198</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" s="1">
         <v>226</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" s="1">
         <v>254</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" s="1">
         <v>282</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" s="1">
         <v>310</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" s="1">
         <v>338</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" s="1">
         <v>366</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" s="1">
         <v>394</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A90" s="1">
         <v>422</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A91" s="1">
         <v>450</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>135</v>
       </c>
     </row>
@@ -2006,6 +2009,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002AA8BEAC825CAE4DA772B4C276EF423C" ma:contentTypeVersion="12" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="4363adfface29496c4692934bfc386e4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="568ff3df-f16a-482d-bb3c-58af1efa1658" xmlns:ns3="13cea704-446d-46be-be94-9e10425fef80" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5ef7a87983d964890dd86635184f037c" ns2:_="" ns3:_="">
     <xsd:import namespace="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
@@ -2216,15 +2228,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2236,13 +2239,38 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41158AEF-3118-4275-B45E-292D0EB8FEF9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55270B5A-DA37-4169-935D-6AA75B2350C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55270B5A-DA37-4169-935D-6AA75B2350C3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41158AEF-3118-4275-B45E-292D0EB8FEF9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
+    <ds:schemaRef ds:uri="13cea704-446d-46be-be94-9e10425fef80"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67DBA8F4-3B6A-4B60-8AA0-23529ABE22D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67DBA8F4-3B6A-4B60-8AA0-23529ABE22D5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>